<commit_message>
pipeline run: 16 businesses found at residential arnona addresses (idx 592-7783)
Searched addresses from index 592 to 7783, covering streets from אבינדב
through בורלא יהודה. Found 16 businesses at residential arnona addresses
including law offices, accountants, clinics, and service businesses.

Progress: __PROGRESS__idx7783.txt

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEy9KWeS2o5FJsz5Murjwg
</commit_message>
<xml_diff>
--- a/reports/דוח נכסים חשודים 03.07.2026.xlsx
+++ b/reports/דוח נכסים חשודים 03.07.2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="עסקים חשודים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="דוח נכסים חשודים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,14 +35,8 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000563C1"/>
-      <sz val="10"/>
-      <u val="single"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,16 +46,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D6E4F0"/>
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -74,39 +65,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="001F4E79"/>
-      </left>
-      <right style="thin">
-        <color rgb="001F4E79"/>
-      </right>
-      <top style="thin">
-        <color rgb="001F4E79"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="001F4E79"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -473,19 +450,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
     <col width="50" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -540,20 +517,20 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1">
+    <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>אבו ננה אחמד</t>
+          <t>מרכז לשרותי בריאות וקהילה</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>בניית בתים חד-משפחתיים</t>
+          <t>קופת חולים / שירותי בריאות</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>אבו זיד אל-הילאל 11</t>
+          <t>אבינדב 2</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -563,7 +540,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>אבו זיד אל-הילאל 11</t>
+          <t>אבינדב 2</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -584,72 +561,72 @@
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>https://www.dunsguide.co.il/Cb9c55068b6a5e8f2cdb2157b2dbd1a38_%D7%97%D7%91%D7%A8%D7%95%D7%AA_%D7%91%D7%A0%D7%99%D7%94_%D7%95%D7%A0%D7%93%D7%9C%D7%9F/%D7%90%D7%91%D7%95_%D7%A0%D7%A0%D7%94_%D7%90%D7%97%D7%9E%D7%93</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="40" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>אלקצאר שירות בריאות בע"מ</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>מרפאה עצמאית</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>אבו רביע 18</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>אבו רביע 18</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>https://www.clalit.co.il/he/sefersherut/pages/clinicdetails.aspx?ddeptcode=14630</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
+          <t>https://www.d.co.il/21355490/32060</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>מרפאה משה הופמן תרפיות</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>מרפאה / פיזיותרפיה</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>אבינועם ילין 13</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>אבינועם ילין 13</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.clalit.co.il/he/sefersherut/pages/doctordetails.aspx?edeptcode=988052269&amp;eservicecode=161000&amp;employeeid=BCCB8A3341815823F3E8410EBE0E7EC5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>אל אקצא - בית מרקחת</t>
+          <t>לאומית שירותי בריאות ירושלים</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>בית מרקחת</t>
+          <t>קופת חולים</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>אבו רביע 18</t>
+          <t>אביתר הכהן 1</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -659,7 +636,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>אבו רביע 18</t>
+          <t>אביתר הכהן 1</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -680,72 +657,72 @@
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>https://www.clalit.co.il/he/sefersherut/pages/pharmacydetails.aspx?ddeptcode=19075</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>האחים קליניס בע"מ</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>ניקיון משרדים</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>אבולעפיה 2</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>אבולעפיה 2</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>https://www.dunsguide.co.il/Ccb515ad66658baa565d2d5e40b70eca4_%D7%A0%D7%99%D7%A7%D7%99%D7%95%D7%9F_%D7%9E%D7%A9%D7%A8%D7%93%D7%99%D7%9D/%D7%94%D7%90%D7%97%D7%99%D7%9D_%D7%A7%D7%9C%D7%99%D7%A0%D7%99%D7%A1</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+          <t>https://www.d.co.il/34212600/43950</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>דניאל קאהן - מעסה רפואי בכיר</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>טיפול גוף / רפואה משלימה</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>אבן שמואל 37</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>אבן שמואל 37</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80364123/40030046</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>עובד - שרותי ניקיון בע"מ</t>
+          <t>רון הרן</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ניקיון משרדים</t>
+          <t>משרד פרסום</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>אבולעפיה 2</t>
+          <t>אבן שפרוט 16</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -755,7 +732,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>אבולעפיה 2</t>
+          <t>אבן שפרוט 16</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -776,67 +753,539 @@
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>https://www.dunsguide.co.il/C806a38831371870e93d1685b9caa4764_%D7%A0%D7%99%D7%A7%D7%99%D7%95%D7%9F_%D7%9E%D7%A9%D7%A8%D7%93%D7%99%D7%9D/%D7%A2%D7%95%D7%91%D7%93_%D7%A9%D7%A8%D7%95%D7%AA%D7%99_%D7%A0%D7%99%D7%A7%D7%99%D7%95%D7%9F</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>שטרודל נקודה קום בע"מ</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>חברות היי-טק ומחשוב</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>אבולעפיה 30</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>אבולעפיה 30</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>https://www.dunsguide.co.il/C66930156e7ddd847edf910e6deaa2f0f_%D7%97%D7%91%D7%A8%D7%95%D7%AA_%D7%94%D7%99%D7%98%D7%A7_%D7%95%D7%9E%D7%99%D7%97%D7%A9%D7%95%D7%91/%D7%A9%D7%98%D7%A8%D7%95%D7%93%D7%9C_%D7%A0%D7%A7%D7%95%D7%93%D7%94_%D7%A7%D7%95%D7%9D</t>
+          <t>https://www.dunsguide.co.il/Ca084ce5b1147b3832bee5cdafa9cca9a_%D7%9E%D7%A9%D7%A8%D7%93%D7%99_%D7%A4%D7%A8%D7%A1%D7%95%D7%9D/%D7%A8%D7%95%D7%9F_%D7%94%D7%A8%D7%9F</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>פוגל יורם</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>אדריכלים</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>אבן שפרוט 16</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>אבן שפרוט 16</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/6018720/630</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>אפשטיין ושות' משרד עו"ד</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>משרד עורכי דין</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 28</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 28</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80256202/9010118</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>זילברמן אליעזר</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>משרד רואי חשבון</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 9</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 9</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/16448300/46140</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>משכן לבטח בע"מ</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>שיפוצים ותיקונים</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 35</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>אלפסי 35</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80314169/48570</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>עומר געש</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>גרפיקאים / עיצוב</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ארלוזורוב 5</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>ארלוזורוב 5</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80070036/11301</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>גנענע</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>שירותי גינון</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 12</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 12</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80010504/11000</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>נגיעה בעץ</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>פרגולות / נגרות</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 22</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 22</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80163803/40480</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>חשמל עמיהוד</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>חשמלאים</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 30</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 30</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80029577/17910</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>פולישוק דניאל - ייעוץ בנקאי</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ייעוץ פיננסי / בנקאי</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 58</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 58</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/80336727/19770</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ד"ר פליישמן צבי</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>מרפאה וטרינרית</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 60</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 60</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/33125270/14670</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>נגיעה בעץ</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>פרגולות / נגרות</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 60</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>גבוה</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>בורוכוב 60</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>נמצא בחיפוש אינטרנט בכתובת מגורים ממרשימת הארנונה</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.d.co.il/64276600/40480</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J7" r:id="rId6"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>